<commit_message>
refactor: substrate helpers, smoother, spectral preproc + examples et rapport
</commit_message>
<xml_diff>
--- a/example/exemple_substrate_index/exemple_substrate_index.xlsx
+++ b/example/exemple_substrate_index/exemple_substrate_index.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lemarchand\Mon Drive\couches minces 2026\CERTUS\2605\example\exemple_substrate_index\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBDB150-8043-4F96-917D-A47C4BB2B8D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="21880" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="measurement" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -28,8 +34,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -66,13 +72,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -110,7 +124,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -144,6 +158,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -178,9 +193,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -353,11 +369,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C51"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="25.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -368,42 +387,42 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>400</v>
       </c>
       <c r="B2">
-        <v>84.55500000000001</v>
+        <v>84.555000000000007</v>
       </c>
       <c r="C2">
         <v>15.445</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>410.204</v>
+        <v>410.20400000000001</v>
       </c>
       <c r="B3">
-        <v>84.46599999999999</v>
+        <v>84.465999999999994</v>
       </c>
       <c r="C3">
-        <v>15.534</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+        <v>15.534000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>420.408</v>
+        <v>420.40800000000002</v>
       </c>
       <c r="B4">
-        <v>84.93899999999999</v>
+        <v>84.938999999999993</v>
       </c>
       <c r="C4">
         <v>15.061</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>430.612</v>
+        <v>430.61200000000002</v>
       </c>
       <c r="B5">
         <v>85</v>
@@ -412,9 +431,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>440.816</v>
+        <v>440.81599999999997</v>
       </c>
       <c r="B6">
         <v>84.738</v>
@@ -423,20 +442,20 @@
         <v>15.262</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>451.02</v>
       </c>
       <c r="B7">
-        <v>84.983</v>
+        <v>84.983000000000004</v>
       </c>
       <c r="C7">
-        <v>15.017</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+        <v>15.016999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>461.224</v>
+        <v>461.22399999999999</v>
       </c>
       <c r="B8">
         <v>85</v>
@@ -445,9 +464,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9">
-        <v>471.429</v>
+        <v>471.42899999999997</v>
       </c>
       <c r="B9">
         <v>85</v>
@@ -456,9 +475,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10">
-        <v>481.633</v>
+        <v>481.63299999999998</v>
       </c>
       <c r="B10">
         <v>85</v>
@@ -467,9 +486,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11">
-        <v>491.837</v>
+        <v>491.83699999999999</v>
       </c>
       <c r="B11">
         <v>85</v>
@@ -478,7 +497,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>502.041</v>
       </c>
@@ -489,7 +508,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>512.245</v>
       </c>
@@ -500,9 +519,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14">
-        <v>522.449</v>
+        <v>522.44899999999996</v>
       </c>
       <c r="B14">
         <v>85</v>
@@ -511,9 +530,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15">
-        <v>532.653</v>
+        <v>532.65300000000002</v>
       </c>
       <c r="B15">
         <v>85</v>
@@ -522,9 +541,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16">
-        <v>542.857</v>
+        <v>542.85699999999997</v>
       </c>
       <c r="B16">
         <v>85</v>
@@ -533,9 +552,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17">
-        <v>553.061</v>
+        <v>553.06100000000004</v>
       </c>
       <c r="B17">
         <v>85</v>
@@ -544,9 +563,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18">
-        <v>563.265</v>
+        <v>563.26499999999999</v>
       </c>
       <c r="B18">
         <v>85</v>
@@ -555,9 +574,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19">
-        <v>573.4690000000001</v>
+        <v>573.46900000000005</v>
       </c>
       <c r="B19">
         <v>85</v>
@@ -566,7 +585,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>583.673</v>
       </c>
@@ -577,9 +596,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21">
-        <v>593.878</v>
+        <v>593.87800000000004</v>
       </c>
       <c r="B21">
         <v>85</v>
@@ -588,9 +607,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22">
-        <v>604.082</v>
+        <v>604.08199999999999</v>
       </c>
       <c r="B22">
         <v>85</v>
@@ -599,18 +618,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23">
-        <v>614.2859999999999</v>
+        <v>614.28599999999994</v>
       </c>
       <c r="B23">
-        <v>84.898</v>
+        <v>84.897999999999996</v>
       </c>
       <c r="C23">
         <v>15.102</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>624.49</v>
       </c>
@@ -621,20 +640,20 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25">
-        <v>634.694</v>
+        <v>634.69399999999996</v>
       </c>
       <c r="B25">
-        <v>84.702</v>
+        <v>84.701999999999998</v>
       </c>
       <c r="C25">
         <v>15.298</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26">
-        <v>644.898</v>
+        <v>644.89800000000002</v>
       </c>
       <c r="B26">
         <v>84.5</v>
@@ -643,9 +662,9 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27">
-        <v>655.102</v>
+        <v>655.10199999999998</v>
       </c>
       <c r="B27">
         <v>84.36</v>
@@ -654,9 +673,9 @@
         <v>15.64</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28">
-        <v>665.306</v>
+        <v>665.30600000000004</v>
       </c>
       <c r="B28">
         <v>84.366</v>
@@ -665,249 +684,249 @@
         <v>15.634</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>675.51</v>
       </c>
       <c r="B29">
-        <v>84.188</v>
+        <v>84.188000000000002</v>
       </c>
       <c r="C29">
-        <v>15.812</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
+        <v>15.811999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30">
-        <v>685.7140000000001</v>
+        <v>685.71400000000006</v>
       </c>
       <c r="B30">
-        <v>84.054</v>
+        <v>84.054000000000002</v>
       </c>
       <c r="C30">
         <v>15.946</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31">
-        <v>695.918</v>
+        <v>695.91800000000001</v>
       </c>
       <c r="B31">
-        <v>83.923</v>
+        <v>83.923000000000002</v>
       </c>
       <c r="C31">
-        <v>16.077</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
+        <v>16.077000000000002</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32">
-        <v>706.122</v>
+        <v>706.12199999999996</v>
       </c>
       <c r="B32">
-        <v>84.108</v>
+        <v>84.108000000000004</v>
       </c>
       <c r="C32">
-        <v>15.892</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
+        <v>15.891999999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>716.327</v>
       </c>
       <c r="B33">
-        <v>83.539</v>
+        <v>83.539000000000001</v>
       </c>
       <c r="C33">
-        <v>16.461</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
+        <v>16.460999999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34">
-        <v>726.5309999999999</v>
+        <v>726.53099999999995</v>
       </c>
       <c r="B34">
-        <v>83.42400000000001</v>
+        <v>83.424000000000007</v>
       </c>
       <c r="C34">
-        <v>16.576</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
+        <v>16.576000000000001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35">
-        <v>736.735</v>
+        <v>736.73500000000001</v>
       </c>
       <c r="B35">
-        <v>83.29000000000001</v>
+        <v>83.29</v>
       </c>
       <c r="C35">
         <v>16.71</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36">
-        <v>746.939</v>
+        <v>746.93899999999996</v>
       </c>
       <c r="B36">
-        <v>83.485</v>
+        <v>83.484999999999999</v>
       </c>
       <c r="C36">
-        <v>16.515</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
+        <v>16.515000000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37">
-        <v>757.143</v>
+        <v>757.14300000000003</v>
       </c>
       <c r="B37">
-        <v>83.533</v>
+        <v>83.533000000000001</v>
       </c>
       <c r="C37">
-        <v>16.467</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
+        <v>16.466999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38">
-        <v>767.347</v>
+        <v>767.34699999999998</v>
       </c>
       <c r="B38">
-        <v>83.285</v>
+        <v>83.284999999999997</v>
       </c>
       <c r="C38">
         <v>16.715</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39">
-        <v>777.551</v>
+        <v>777.55100000000004</v>
       </c>
       <c r="B39">
-        <v>83.149</v>
+        <v>83.149000000000001</v>
       </c>
       <c r="C39">
-        <v>16.851</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
+        <v>16.850999999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>787.755</v>
       </c>
       <c r="B40">
-        <v>83.167</v>
+        <v>83.167000000000002</v>
       </c>
       <c r="C40">
-        <v>16.833</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
+        <v>16.832999999999998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41">
-        <v>797.9589999999999</v>
+        <v>797.95899999999995</v>
       </c>
       <c r="B41">
-        <v>83.467</v>
+        <v>83.466999999999999</v>
       </c>
       <c r="C41">
-        <v>16.533</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
+        <v>16.533000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42">
-        <v>808.163</v>
+        <v>808.16300000000001</v>
       </c>
       <c r="B42">
-        <v>83.536</v>
+        <v>83.536000000000001</v>
       </c>
       <c r="C42">
-        <v>16.464</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
+        <v>16.463999999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43">
-        <v>818.367</v>
+        <v>818.36699999999996</v>
       </c>
       <c r="B43">
-        <v>83.572</v>
+        <v>83.572000000000003</v>
       </c>
       <c r="C43">
-        <v>16.428</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
+        <v>16.428000000000001</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44">
-        <v>828.571</v>
+        <v>828.57100000000003</v>
       </c>
       <c r="B44">
-        <v>83.44199999999999</v>
+        <v>83.441999999999993</v>
       </c>
       <c r="C44">
         <v>16.558</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45">
-        <v>838.776</v>
+        <v>838.77599999999995</v>
       </c>
       <c r="B45">
-        <v>83.70699999999999</v>
+        <v>83.706999999999994</v>
       </c>
       <c r="C45">
-        <v>16.293</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
+        <v>16.292999999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>848.98</v>
       </c>
       <c r="B46">
-        <v>83.803</v>
+        <v>83.802999999999997</v>
       </c>
       <c r="C46">
-        <v>16.197</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
+        <v>16.196999999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47">
-        <v>859.184</v>
+        <v>859.18399999999997</v>
       </c>
       <c r="B47">
-        <v>83.95099999999999</v>
+        <v>83.950999999999993</v>
       </c>
       <c r="C47">
-        <v>16.049</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
+        <v>16.048999999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48">
-        <v>869.388</v>
+        <v>869.38800000000003</v>
       </c>
       <c r="B48">
-        <v>84.20699999999999</v>
+        <v>84.206999999999994</v>
       </c>
       <c r="C48">
-        <v>15.793</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
+        <v>15.792999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49">
-        <v>879.592</v>
+        <v>879.59199999999998</v>
       </c>
       <c r="B49">
-        <v>84.236</v>
+        <v>84.236000000000004</v>
       </c>
       <c r="C49">
-        <v>15.764</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
+        <v>15.763999999999999</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50">
-        <v>889.796</v>
+        <v>889.79600000000005</v>
       </c>
       <c r="B50">
-        <v>84.46899999999999</v>
+        <v>84.468999999999994</v>
       </c>
       <c r="C50">
-        <v>15.531</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3">
+        <v>15.531000000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>900</v>
       </c>

</xml_diff>